<commit_message>
Add notification, translation and push-ups items to roadmap
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Fz4xPsgT9AKmio7bR21oo1
</commit_message>
<xml_diff>
--- a/docs/habitt_roadmap.xlsx
+++ b/docs/habitt_roadmap.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Roadmap!$A$5:$J$30</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Roadmap!$A$5:$J$34</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="132">
   <si>
     <t xml:space="preserve">Habitt v2: Feature &amp; Fix Backlog (easiest to hardest)</t>
   </si>
@@ -140,6 +140,21 @@
     <t xml:space="preserve">Mostly handled in commit 063d2bd (HabitRouteTracker + _navigateToHabit replaces the page). Reproduce to find any edge case that is left, e.g. a details page opened from another route.</t>
   </si>
   <si>
+    <t xml:space="preserve">Add missing translations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Localization</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Your list (17.10.)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Translate the strings that exist in English but are missing in the other languages.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">94 keys are missing in each of app_bs/de/es/it.arb (en has them). Copy work + gen-l10n; low risk.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Fix: streak wrong after completing a past day then today (amount/optional habits)</t>
   </si>
   <si>
@@ -185,6 +200,15 @@
     <t xml:space="preserve">README says the logic exists (e.g. Habit.getStartHour); only UI needed.</t>
   </si>
   <si>
+    <t xml:space="preserve">Fix: push-ups notification shows a whole list of texts instead of one chosen text</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The push-ups habit notification shows all text variants together instead of picking one.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Push-ups is not a premade type in premade_habit_type.dart, so it likely hits a generic/fallback path in services/notification_text (composer / template_catalog). Needs a repro to find where the list gets joined.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Time counter: how long you've been doing a habit + strength graph over time</t>
   </si>
   <si>
@@ -219,6 +243,27 @@
   </si>
   <si>
     <t xml:space="preserve">lib/util/insight_sheet_flow.dart currently shows sheets one at a time (debounced). Needs a refactor to collect and batch them.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tapping a notification opens the Log progress dialog instead of habit details</t>
+  </si>
+  <si>
+    <t xml:space="preserve">For amount/duration habits, tapping the notification opens log_progress_dialog to enter progress right away.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Change _navigateToHabit in notification_action_handler.dart. Needs a cold-start path (dialog after the navigator is ready), a rule for checkbox habits (keep details page or complete), and the right day selected.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Improve notification texts in general</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Notifications</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rewrite and expand notification copy so it's more varied, natural and motivating, in all 5 languages.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Text system is in services/notification_text (composer, template_catalog, rules/). Overlaps with README #4, so do them together. Effort is mostly writing + translating.</t>
   </si>
   <si>
     <t xml:space="preserve">Habit goals (README #1)</t>
@@ -1008,7 +1053,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J30"/>
+  <dimension ref="A1:J34"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -1242,7 +1287,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="n">
         <v>6</v>
       </c>
@@ -1250,19 +1295,19 @@
         <v>38</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H11" s="12" t="s">
         <v>29</v>
@@ -1272,24 +1317,24 @@
         <v>19</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="n">
         <v>7</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>15</v>
+        <v>44</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="G12" s="5" t="n">
         <v>3</v>
@@ -1307,7 +1352,7 @@
         <v>8</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C13" s="6" t="s">
         <v>14</v>
@@ -1316,10 +1361,10 @@
         <v>15</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="G13" s="5" t="n">
         <v>3</v>
@@ -1337,13 +1382,13 @@
         <v>9</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>49</v>
+        <v>14</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>50</v>
+        <v>15</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>51</v>
@@ -1370,40 +1415,40 @@
         <v>53</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G15" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="H15" s="13" t="s">
-        <v>57</v>
+        <v>3</v>
+      </c>
+      <c r="H15" s="12" t="s">
+        <v>29</v>
       </c>
       <c r="I15" s="8"/>
       <c r="J15" s="5" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="9" t="n">
+    <row r="16" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="5" t="n">
         <v>11</v>
       </c>
-      <c r="B16" s="10" t="s">
+      <c r="B16" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="C16" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="D16" s="10" t="s">
-        <v>15</v>
+      <c r="C16" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>40</v>
       </c>
       <c r="E16" s="6" t="s">
         <v>59</v>
@@ -1412,14 +1457,12 @@
         <v>60</v>
       </c>
       <c r="G16" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="H16" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="I16" s="11" t="s">
-        <v>24</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="H16" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="I16" s="8"/>
       <c r="J16" s="5" t="s">
         <v>19</v>
       </c>
@@ -1432,10 +1475,10 @@
         <v>61</v>
       </c>
       <c r="C17" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="D17" s="6" t="s">
         <v>62</v>
-      </c>
-      <c r="D17" s="6" t="s">
-        <v>15</v>
       </c>
       <c r="E17" s="6" t="s">
         <v>63</v>
@@ -1447,7 +1490,7 @@
         <v>4</v>
       </c>
       <c r="H17" s="13" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="I17" s="8"/>
       <c r="J17" s="5" t="s">
@@ -1455,91 +1498,91 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="5" t="n">
+      <c r="A18" s="9" t="n">
         <v>13</v>
       </c>
-      <c r="B18" s="6" t="s">
+      <c r="B18" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="C18" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="D18" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="E18" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="G18" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="H18" s="13" t="s">
         <v>65</v>
       </c>
-      <c r="C18" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="D18" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="E18" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="F18" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="G18" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="H18" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="I18" s="8"/>
+      <c r="I18" s="11" t="s">
+        <v>24</v>
+      </c>
       <c r="J18" s="5" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="9" t="n">
+    <row r="19" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="5" t="n">
         <v>14</v>
       </c>
-      <c r="B19" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="C19" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="D19" s="10" t="s">
+      <c r="B19" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="D19" s="6" t="s">
         <v>15</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G19" s="5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H19" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="I19" s="11" t="s">
-        <v>24</v>
-      </c>
+        <v>65</v>
+      </c>
+      <c r="I19" s="8"/>
       <c r="J19" s="5" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="n">
         <v>15</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="G20" s="5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H20" s="13" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="I20" s="8"/>
       <c r="J20" s="5" t="s">
@@ -1551,25 +1594,25 @@
         <v>16</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>49</v>
+        <v>77</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="G21" s="5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H21" s="13" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="I21" s="8"/>
       <c r="J21" s="5" t="s">
@@ -1581,57 +1624,59 @@
         <v>17</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="G22" s="5" t="n">
         <v>5</v>
       </c>
       <c r="H22" s="13" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="I22" s="8"/>
       <c r="J22" s="5" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="5" t="n">
+    <row r="23" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="9" t="n">
         <v>18</v>
       </c>
-      <c r="B23" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="C23" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="D23" s="6" t="s">
+      <c r="B23" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="C23" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="D23" s="10" t="s">
         <v>15</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="G23" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="H23" s="14" t="s">
-        <v>83</v>
-      </c>
-      <c r="I23" s="8"/>
+        <v>5</v>
+      </c>
+      <c r="H23" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="I23" s="11" t="s">
+        <v>24</v>
+      </c>
       <c r="J23" s="5" t="s">
         <v>19</v>
       </c>
@@ -1641,73 +1686,73 @@
         <v>19</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>49</v>
+        <v>70</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>85</v>
+        <v>15</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="G24" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="H24" s="14" t="s">
-        <v>83</v>
+        <v>5</v>
+      </c>
+      <c r="H24" s="13" t="s">
+        <v>65</v>
       </c>
       <c r="I24" s="8"/>
       <c r="J24" s="5" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="n">
         <v>20</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="F25" s="6" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="G25" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="H25" s="14" t="s">
-        <v>83</v>
+        <v>5</v>
+      </c>
+      <c r="H25" s="13" t="s">
+        <v>65</v>
       </c>
       <c r="I25" s="8"/>
       <c r="J25" s="5" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="9" t="n">
+    <row r="26" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="5" t="n">
         <v>21</v>
       </c>
-      <c r="B26" s="10" t="s">
-        <v>91</v>
-      </c>
-      <c r="C26" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="D26" s="10" t="s">
+      <c r="B26" s="6" t="s">
         <v>92</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>55</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>93</v>
@@ -1716,19 +1761,17 @@
         <v>94</v>
       </c>
       <c r="G26" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="H26" s="14" t="s">
-        <v>83</v>
-      </c>
-      <c r="I26" s="11" t="s">
-        <v>24</v>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="H26" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="I26" s="8"/>
       <c r="J26" s="5" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="n">
         <v>22</v>
       </c>
@@ -1736,10 +1779,10 @@
         <v>95</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>49</v>
+        <v>70</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>54</v>
+        <v>15</v>
       </c>
       <c r="E27" s="6" t="s">
         <v>96</v>
@@ -1748,47 +1791,47 @@
         <v>97</v>
       </c>
       <c r="G27" s="5" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H27" s="14" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="I27" s="8"/>
       <c r="J27" s="5" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="n">
         <v>23</v>
       </c>
       <c r="B28" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="D28" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="E28" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="F28" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="G28" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="H28" s="14" t="s">
         <v>98</v>
-      </c>
-      <c r="C28" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="D28" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="E28" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="F28" s="6" t="s">
-        <v>101</v>
-      </c>
-      <c r="G28" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="H28" s="15" t="s">
-        <v>102</v>
       </c>
       <c r="I28" s="8"/>
       <c r="J28" s="5" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="n">
         <v>24</v>
       </c>
@@ -1796,10 +1839,10 @@
         <v>103</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>99</v>
+        <v>54</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>85</v>
+        <v>55</v>
       </c>
       <c r="E29" s="6" t="s">
         <v>104</v>
@@ -1808,54 +1851,176 @@
         <v>105</v>
       </c>
       <c r="G29" s="5" t="n">
-        <v>9</v>
-      </c>
-      <c r="H29" s="15" t="s">
-        <v>102</v>
+        <v>7</v>
+      </c>
+      <c r="H29" s="14" t="s">
+        <v>98</v>
       </c>
       <c r="I29" s="8"/>
       <c r="J29" s="5" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="5" t="n">
+    <row r="30" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="9" t="n">
         <v>25</v>
       </c>
-      <c r="B30" s="6" t="s">
+      <c r="B30" s="10" t="s">
         <v>106</v>
       </c>
-      <c r="C30" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="D30" s="6" t="s">
+      <c r="C30" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="D30" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="E30" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="F30" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="G30" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="H30" s="14" t="s">
+        <v>98</v>
+      </c>
+      <c r="I30" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="J30" s="5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="5" t="n">
         <v>26</v>
       </c>
-      <c r="E30" s="6" t="s">
-        <v>107</v>
-      </c>
-      <c r="F30" s="6" t="s">
-        <v>108</v>
-      </c>
-      <c r="G30" s="5" t="n">
+      <c r="B31" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="D31" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="E31" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="F31" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="G31" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="H31" s="14" t="s">
+        <v>98</v>
+      </c>
+      <c r="I31" s="8"/>
+      <c r="J31" s="5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="5" t="n">
+        <v>27</v>
+      </c>
+      <c r="B32" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="D32" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="E32" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="F32" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="G32" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="H32" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="I32" s="8"/>
+      <c r="J32" s="5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="D33" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="E33" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="F33" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="G33" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="H33" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="I33" s="8"/>
+      <c r="J33" s="5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="5" t="n">
+        <v>29</v>
+      </c>
+      <c r="B34" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="C34" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="D34" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="E34" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="F34" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="G34" s="5" t="n">
         <v>10</v>
       </c>
-      <c r="H30" s="15" t="s">
-        <v>102</v>
-      </c>
-      <c r="I30" s="8"/>
-      <c r="J30" s="5" t="s">
+      <c r="H34" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="I34" s="8"/>
+      <c r="J34" s="5" t="s">
         <v>19</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:J30"/>
+  <autoFilter ref="A5:J34"/>
   <mergeCells count="2">
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="A3:I3"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J6:J30" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J6:J34" type="list">
       <formula1>"To do,In progress,Done,Verify"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -1886,7 +2051,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>109</v>
+        <v>124</v>
       </c>
       <c r="B1" s="16"/>
       <c r="C1" s="16"/>
@@ -1901,10 +2066,10 @@
         <v>10</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>110</v>
+        <v>125</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>111</v>
+        <v>126</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1912,11 +2077,11 @@
         <v>18</v>
       </c>
       <c r="B4" s="16" t="n">
-        <f aca="false">COUNTIF(Roadmap!$H$6:$H$30,A4)</f>
+        <f aca="false">COUNTIF(Roadmap!$H$6:$H$34,A4)</f>
         <v>2</v>
       </c>
       <c r="C4" s="16" t="n">
-        <f aca="false">COUNTIFS(Roadmap!$H$6:$H$30,A4,Roadmap!$J$6:$J$30,"Done")</f>
+        <f aca="false">COUNTIFS(Roadmap!$H$6:$H$34,A4,Roadmap!$J$6:$J$34,"Done")</f>
         <v>0</v>
       </c>
     </row>
@@ -1925,60 +2090,60 @@
         <v>29</v>
       </c>
       <c r="B5" s="16" t="n">
-        <f aca="false">COUNTIF(Roadmap!$H$6:$H$30,A5)</f>
-        <v>7</v>
+        <f aca="false">COUNTIF(Roadmap!$H$6:$H$34,A5)</f>
+        <v>9</v>
       </c>
       <c r="C5" s="16" t="n">
-        <f aca="false">COUNTIFS(Roadmap!$H$6:$H$30,A5,Roadmap!$J$6:$J$30,"Done")</f>
+        <f aca="false">COUNTIFS(Roadmap!$H$6:$H$34,A5,Roadmap!$J$6:$J$34,"Done")</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="20" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="B6" s="16" t="n">
-        <f aca="false">COUNTIF(Roadmap!$H$6:$H$30,A6)</f>
-        <v>8</v>
+        <f aca="false">COUNTIF(Roadmap!$H$6:$H$34,A6)</f>
+        <v>10</v>
       </c>
       <c r="C6" s="16" t="n">
-        <f aca="false">COUNTIFS(Roadmap!$H$6:$H$30,A6,Roadmap!$J$6:$J$30,"Done")</f>
+        <f aca="false">COUNTIFS(Roadmap!$H$6:$H$34,A6,Roadmap!$J$6:$J$34,"Done")</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="21" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="B7" s="16" t="n">
-        <f aca="false">COUNTIF(Roadmap!$H$6:$H$30,A7)</f>
+        <f aca="false">COUNTIF(Roadmap!$H$6:$H$34,A7)</f>
         <v>5</v>
       </c>
       <c r="C7" s="16" t="n">
-        <f aca="false">COUNTIFS(Roadmap!$H$6:$H$30,A7,Roadmap!$J$6:$J$30,"Done")</f>
+        <f aca="false">COUNTIFS(Roadmap!$H$6:$H$34,A7,Roadmap!$J$6:$J$34,"Done")</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="22" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="B8" s="16" t="n">
-        <f aca="false">COUNTIF(Roadmap!$H$6:$H$30,A8)</f>
+        <f aca="false">COUNTIF(Roadmap!$H$6:$H$34,A8)</f>
         <v>3</v>
       </c>
       <c r="C8" s="16" t="n">
-        <f aca="false">COUNTIFS(Roadmap!$H$6:$H$30,A8,Roadmap!$J$6:$J$30,"Done")</f>
+        <f aca="false">COUNTIFS(Roadmap!$H$6:$H$34,A8,Roadmap!$J$6:$J$34,"Done")</f>
         <v>0</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="23" t="s">
-        <v>112</v>
+        <v>127</v>
       </c>
       <c r="B9" s="16" t="n">
         <f aca="false">SUM(B4:B8)</f>
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="C9" s="16" t="n">
         <f aca="false">SUM(C4:C8)</f>
@@ -1992,20 +2157,20 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="23" t="s">
-        <v>113</v>
+        <v>128</v>
       </c>
       <c r="B11" s="16" t="n">
-        <f aca="false">COUNTIF(Roadmap!$I$6:$I$30,"YES")</f>
+        <f aca="false">COUNTIF(Roadmap!$I$6:$I$34,"YES")</f>
         <v>6</v>
       </c>
       <c r="C11" s="16" t="n">
-        <f aca="false">COUNTIFS(Roadmap!$I$6:$I$30,"YES",Roadmap!$J$6:$J$30,"Done")</f>
+        <f aca="false">COUNTIFS(Roadmap!$I$6:$I$34,"YES",Roadmap!$J$6:$J$34,"Done")</f>
         <v>0</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="23" t="s">
-        <v>114</v>
+        <v>129</v>
       </c>
       <c r="B12" s="16" t="str">
         <f aca="false">IF(C11=B11,"YES - can publish","NO - finish Health sync first")</f>
@@ -2020,14 +2185,14 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="16" t="s">
-        <v>115</v>
+        <v>130</v>
       </c>
       <c r="B14" s="16"/>
       <c r="C14" s="16"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="16" t="s">
-        <v>116</v>
+        <v>131</v>
       </c>
       <c r="B15" s="16"/>
       <c r="C15" s="16"/>

</xml_diff>

<commit_message>
Roadmap: checkbox habits keep opening details on notification tap
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Fz4xPsgT9AKmio7bR21oo1
</commit_message>
<xml_diff>
--- a/docs/habitt_roadmap.xlsx
+++ b/docs/habitt_roadmap.xlsx
@@ -248,10 +248,10 @@
     <t xml:space="preserve">Tapping a notification opens the Log progress dialog instead of habit details</t>
   </si>
   <si>
-    <t xml:space="preserve">For amount/duration habits, tapping the notification opens log_progress_dialog to enter progress right away.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Change _navigateToHabit in notification_action_handler.dart. Needs a cold-start path (dialog after the navigator is ready), a rule for checkbox habits (keep details page or complete), and the right day selected.</t>
+    <t xml:space="preserve">Amount/duration habits: tapping the notification opens log_progress_dialog to enter progress right away. Checkbox habits: open the habit details page (as now).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Change _navigateToHabit in notification_action_handler.dart. Needs a cold-start path (dialog after the navigator is ready) and the right day selected. Decided: checkbox habits keep opening the details page.</t>
   </si>
   <si>
     <t xml:space="preserve">Improve notification texts in general</t>

</xml_diff>